<commit_message>
Cronograma integrado CPF2 v2: premisas FAT conjunto + recableado HIMA + flujo temporal HTML
Nuevas premisas:
- HIMA: recepcion en Inauco 26 sem desde 1-AGO -> 30-ENE-2027; nuevo item Recableado
  interno (45 d) 30-ENE->16-MAR que habilita la FAT SIS.
- FAT como prueba conjunta: FAT PCS+Comms confluye en FAT SIS; el FIN FAT integral
  cierra con el sistema mas tardio -> 06-ABR-2027 (nuevo hito).
- Integracion PCS<->PMS reubicada dentro del periodo FAT (no critica).
- Actualizado Gantt PDF, Flujo PDF y XLSX.
- HTML: datos y KPIs actualizados + nueva pestana 'Flujo temporal' (SVG a escala
  temporal, carriles por provision, hitos, bandas periodo FAT/iFAT y convergencia).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVwGTCmUM8cuHgXLywyxFM
</commit_message>
<xml_diff>
--- a/Constructibilidad/Análisis generados/Cronograma_Integrado_CPF2.xlsx
+++ b/Constructibilidad/Análisis generados/Cronograma_Integrado_CPF2.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FAT PCS + Comunicaciones (Neuquén, 18 d)</t>
+          <t>FAT PCS + Comunicaciones (18 d) — confluye en FAT SIS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1115,17 +1115,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Integración PCS↔PMS ABB (Bs.As., 5 d)</t>
+          <t>Integración PCS↔PMS ABB (5 d, dentro del período FAT)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>27-03-2027</t>
+          <t>24-03-2027</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>02-04-2027</t>
+          <t>30-03-2027</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1135,29 +1135,29 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Inauco — PCS / SCADA / Comunicaciones</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>SAT + Comisionado PCS — campo (55 d)</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>17-04-2027</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>02-07-2027</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Tarea</t>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>★ FIN FAT integral (todos los sistemas — el más tardío)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>06-04-2027</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Hito</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SAT + Comisionado SCADA SIS — campo (100 d)</t>
+          <t>SAT + Comisionado PCS — campo (55 d)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>03-09-2027</t>
+          <t>02-07-2027</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1196,103 +1196,103 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>SAT + Comisionado SCADA SIS — campo (100 d)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>17-04-2027</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>03-09-2027</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Inauco — PCS / SCADA / Comunicaciones</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Prueba MCE + CAO (as-built)</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>04-09-2027</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>22-10-2027</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>HIMA — PSS / SIS (ESD · F&amp;G)</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Fabricación tablero SIS (25 sem desde AGO)</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Fabricación tablero SIS (26 sem desde AGO)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
         <is>
           <t>01-08-2026</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>23-01-2027</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>30-01-2027</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>HIMA — PSS / SIS (ESD · F&amp;G)</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>★ Recepción tablero HIMA en Inauco (23-ENE-2027)</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>23-01-2027</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>★ Recepción tablero HIMA en Inauco (30-ENE-2027)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>30-01-2027</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Hito</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>HIMA — PSS / SIS (ESD · F&amp;G)</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>FAT SIS (HIMA + Inauco, 20 d)</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>27-02-2027</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>26-03-2027</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Tarea</t>
         </is>
       </c>
     </row>
@@ -1304,71 +1304,71 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>Recableado interno HIMA (45 d) — habilita FAT SIS</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>30-01-2027</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>16-03-2027</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>HIMA — PSS / SIS (ESD · F&amp;G)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>FAT SIS (conjunto PCS + SIS, 20 d)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>17-03-2027</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>06-04-2027</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>HIMA — PSS / SIS (ESD · F&amp;G)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>Soporte HIMA en campo (SAT/PEM SCADA SIS)</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>17-04-2027</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>03-09-2027</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>Integración EPC (AESA)</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Precomisionado / montaje de campo</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>03-05-2027</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>13-01-2028</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>Integración EPC (AESA)</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>iFAT — Integración Shelters + PMS + INAUCO + HIMA</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>25-06-2027</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>14-07-2027</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1385,17 +1385,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Comisionado</t>
+          <t>Precomisionado / montaje de campo</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16-07-2027</t>
+          <t>03-05-2027</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>31-01-2028</t>
+          <t>13-01-2028</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1412,47 +1412,101 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>iFAT — Integración Shelters + PMS + INAUCO + HIMA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>25-06-2027</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>14-07-2027</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>Integración EPC (AESA)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Comisionado</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>16-07-2027</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>31-01-2028</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>Integración EPC (AESA)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>SAT PMS en sitio (hold point)</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>01-10-2027</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>15-12-2027</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>Integración EPC (AESA)</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>★ RFSU — Ready For Start Up (31-ENE-2028)</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>31-01-2028</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>Hito</t>
         </is>

</xml_diff>